<commit_message>
fix 42 & 删除33 node包
</commit_message>
<xml_diff>
--- a/new-info33/web.xlsx
+++ b/new-info33/web.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="16500" windowHeight="11865"/>
+    <workbookView windowWidth="28800" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="14" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>domain</t>
   </si>
@@ -41,22 +41,13 @@
     <t>color2</t>
   </si>
   <si>
-    <t>xanthium.fun</t>
+    <t>read.xanthium.fun</t>
   </si>
   <si>
     <t>#957aa9</t>
   </si>
   <si>
-    <t>dzos.fun</t>
-  </si>
-  <si>
-    <t>#33325d</t>
-  </si>
-  <si>
-    <t>rorqual.fun</t>
-  </si>
-  <si>
-    <t>#ae1c31</t>
+    <t>sec.xanthium.fun</t>
   </si>
   <si>
     <t>spuddles.fun</t>
@@ -1017,7 +1008,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1085,9 +1076,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1500,6 +1488,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="27.75" customWidth="1"/>
+    <col min="2" max="2" width="13.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1514,56 +1503,52 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="26"/>
+      <c r="C2" s="25"/>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="26"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="26"/>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="B3" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="25"/>
+    </row>
+    <row r="4" ht="15" spans="1:7">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="25"/>
+    </row>
+    <row r="5" ht="15" spans="1:7">
       <c r="A5" s="23"/>
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" ht="15" spans="1:7">
       <c r="A6" s="23"/>
       <c r="B6" s="23"/>
       <c r="C6" s="23"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7">
+      <c r="F17" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="31" t="s">
         <v>9</v>
-      </c>
-      <c r="G16" s="31" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="6:7">
-      <c r="F17" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1571,9 +1556,8 @@
     <hyperlink ref="F16" r:id="rId1" display="spuddles.fun"/>
     <hyperlink ref="F17" r:id="rId2" display="moilfuns.fun"/>
     <hyperlink ref="A6" r:id="rId3" tooltip="https://jentacul.com"/>
-    <hyperlink ref="A2" r:id="rId4" display="xanthium.fun"/>
-    <hyperlink ref="A3" r:id="rId5" display="dzos.fun"/>
-    <hyperlink ref="A4" r:id="rId6" display="rorqual.fun"/>
+    <hyperlink ref="A2" r:id="rId4" display="read.xanthium.fun"/>
+    <hyperlink ref="A3" r:id="rId4" display="sec.xanthium.fun"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1594,27 +1578,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="16" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -1625,13 +1609,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D3" s="15">
         <v>5</v>
@@ -1642,13 +1626,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="16" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D4" s="15">
         <v>3</v>
@@ -1714,27 +1698,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1745,13 +1729,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1804,24 +1788,24 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1832,10 +1816,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1846,10 +1830,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4">

</xml_diff>